<commit_message>
Login--> 2. Deposit Completed
</commit_message>
<xml_diff>
--- a/Bank_Mgmt/bank_records.xlsx
+++ b/Bank_Mgmt/bank_records.xlsx
@@ -1,82 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet sheetId="1" name="Bank Records" state="visible" r:id="rId4"/>
+    <sheet name="Bank Records" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
-  <si>
-    <t>Account No.</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>PIN</t>
-  </si>
-  <si>
-    <t>Transaction ID</t>
-  </si>
-  <si>
-    <t>Transaction Type</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
-    <t>Previous Balance</t>
-  </si>
-  <si>
-    <t>Current Balance</t>
-  </si>
-  <si>
-    <t>Date-Time</t>
-  </si>
-  <si>
-    <t>sid</t>
-  </si>
-  <si>
-    <t>e6737a5d-e</t>
-  </si>
-  <si>
-    <t>Opening</t>
-  </si>
-  <si>
-    <t>2026-09-06 13:39:39</t>
-  </si>
-  <si>
-    <t>amogh</t>
-  </si>
-  <si>
-    <t>c03b69a5-f</t>
-  </si>
-  <si>
-    <t>2026-09-06 13:41:11</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <family val="2"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -95,21 +43,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -434,110 +441,368 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="2" width="13.571428571428571" customWidth="1"/>
-    <col min="3" max="3" width="9.571428571428571" customWidth="1"/>
-    <col min="4" max="4" width="17.285714285714285" customWidth="1"/>
-    <col min="5" max="5" width="19.571428571428573" customWidth="1"/>
-    <col min="6" max="6" width="13.571428571428571" customWidth="1"/>
-    <col min="7" max="7" width="18.142857142857142" customWidth="1"/>
-    <col min="8" max="8" width="16.142857142857142" customWidth="1"/>
-    <col min="9" max="24" width="13.571428571428571" customWidth="1"/>
+    <col width="13.57142857142857" customWidth="1" min="1" max="2"/>
+    <col width="9.571428571428571" customWidth="1" min="3" max="3"/>
+    <col width="17.28571428571428" customWidth="1" min="4" max="4"/>
+    <col width="19.57142857142857" customWidth="1" min="5" max="5"/>
+    <col width="13.57142857142857" customWidth="1" min="6" max="6"/>
+    <col width="18.14285714285714" customWidth="1" min="7" max="7"/>
+    <col width="16.14285714285714" customWidth="1" min="8" max="8"/>
+    <col width="13.57142857142857" customWidth="1" min="9" max="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Account No.</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>PIN</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Transaction ID</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Transaction Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Previous Balance</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Current Balance</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date-Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1234567890</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>sid</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>123456</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>e6737a5d-e</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>123456678</v>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
+      <c r="H2" t="n">
+        <v>123456678</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:39:39</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1234567890</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2">
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1234567891</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>amogh</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>123456</v>
       </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>c03b69a5-f</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>90</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>90</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:41:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sid</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1e73375d-d</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>55000</v>
+      </c>
+      <c r="G4" t="n">
         <v>123456678</v>
       </c>
-      <c r="G2">
+      <c r="H4" t="n">
+        <v>123511678</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:30:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sid</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ce917080-7</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G5" t="n">
+        <v>123456678</v>
+      </c>
+      <c r="H5" t="n">
+        <v>123464678</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:35:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1234567890</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sid</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>76c9d98e-d</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>0</v>
       </c>
-      <c r="H2">
-        <v>123456678</v>
-      </c>
-      <c r="I2" t="s">
-        <v>12</v>
+      <c r="G6" t="n">
+        <v>123511678</v>
+      </c>
+      <c r="H6" t="n">
+        <v>123511678</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-09-11 20:37:47</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1234567891</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3">
-        <v>123456</v>
-      </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1234567891</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>amogh</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>333040b6-a</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>100020</v>
+      </c>
+      <c r="G7" t="n">
         <v>90</v>
       </c>
-      <c r="G3">
+      <c r="H7" t="n">
+        <v>100110</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-09-11 21:16:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2939192033</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dhruv Kale</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>102030</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5d7aaee7-9</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Opening</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G8" t="n">
         <v>0</v>
       </c>
-      <c r="H3">
-        <v>90</v>
-      </c>
-      <c r="I3" t="s">
-        <v>15</v>
+      <c r="H8" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-09-11 21:19:22</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25"/>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2939192033</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dhruv Kale</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>5d5b7afe-7</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Deposit</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="H9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-09-11 21:30:49</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>